<commit_message>
feat(kashmir): corridor de-dup — 104 routes / 670 buses, no duplicate codes
Sync v3.3.8 after corridor-wide consolidation (trunks+feeders). active 133->104,
fleet 817->670 (HPV 76/MPV 550/LPV 44), 0 duplicate route codes/names; coverage
unchanged (31%). Updated lib numbers + synced routes.json/impact.json/workbooks.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.xlsx
+++ b/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.xlsx
@@ -988,7 +988,7 @@
         <v>0.7482</v>
       </c>
       <c r="T2" s="7" t="n">
-        <v>9071</v>
+        <v>11362</v>
       </c>
       <c r="U2" s="7" t="n">
         <v>5.746</v>
@@ -1081,7 +1081,7 @@
         <v>0.0638</v>
       </c>
       <c r="T3" s="7" t="n">
-        <v>8455</v>
+        <v>10590</v>
       </c>
       <c r="U3" s="7" t="n">
         <v>3.4734</v>
@@ -1304,7 +1304,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>FDR-323</t>
+          <t>FDR-320</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D6" s="7" t="n">
@@ -1328,7 +1328,11 @@
       <c r="F6" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
           <t>LP</t>
@@ -1341,7 +1345,7 @@
         <v>113.3</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>0</v>
@@ -1350,7 +1354,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O6" s="7" t="b">
         <v>0</v>
@@ -1362,13 +1366,13 @@
         <v>0.0125</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S6" s="7" t="n">
         <v>0.0638</v>
       </c>
       <c r="T6" s="7" t="n">
-        <v>8455</v>
+        <v>0</v>
       </c>
       <c r="U6" s="7" t="n">
         <v>3.4734</v>
@@ -1461,7 +1465,7 @@
         <v>0.441</v>
       </c>
       <c r="T7" s="7" t="n">
-        <v>9618</v>
+        <v>12048</v>
       </c>
       <c r="U7" s="7" t="n">
         <v>6.8548</v>
@@ -1554,7 +1558,7 @@
         <v>0.2732</v>
       </c>
       <c r="T8" s="7" t="n">
-        <v>16373</v>
+        <v>20509</v>
       </c>
       <c r="U8" s="7" t="n">
         <v>8.305999999999999</v>
@@ -1744,7 +1748,7 @@
         <v>0.7436</v>
       </c>
       <c r="T10" s="7" t="n">
-        <v>9365</v>
+        <v>11731</v>
       </c>
       <c r="U10" s="7" t="n">
         <v>5.422</v>
@@ -1837,7 +1841,7 @@
         <v>0.177</v>
       </c>
       <c r="T11" s="7" t="n">
-        <v>10688</v>
+        <v>13388</v>
       </c>
       <c r="U11" s="7" t="n">
         <v>2.0631</v>
@@ -2027,7 +2031,7 @@
         <v>0.7272</v>
       </c>
       <c r="T13" s="7" t="n">
-        <v>7514</v>
+        <v>9412</v>
       </c>
       <c r="U13" s="7" t="n">
         <v>5.0024</v>
@@ -2056,7 +2060,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>FDR-114</t>
+          <t>FDR-070</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -2066,7 +2070,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D14" s="7" t="n">
@@ -2080,7 +2084,11 @@
       <c r="F14" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
           <t>HP</t>
@@ -2093,7 +2101,7 @@
         <v>86.5</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L14" s="7" t="n">
         <v>0</v>
@@ -2102,7 +2110,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O14" s="7" t="b">
         <v>0</v>
@@ -2114,13 +2122,13 @@
         <v>0.3878</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S14" s="7" t="n">
         <v>0.5865</v>
       </c>
       <c r="T14" s="7" t="n">
-        <v>9863</v>
+        <v>0</v>
       </c>
       <c r="U14" s="7" t="n">
         <v>5.174</v>
@@ -2310,7 +2318,7 @@
         <v>0.5219</v>
       </c>
       <c r="T16" s="7" t="n">
-        <v>10836</v>
+        <v>13574</v>
       </c>
       <c r="U16" s="7" t="n">
         <v>3.5932</v>
@@ -2403,7 +2411,7 @@
         <v>0.527</v>
       </c>
       <c r="T17" s="7" t="n">
-        <v>5985</v>
+        <v>7497</v>
       </c>
       <c r="U17" s="7" t="n">
         <v>3.5833</v>
@@ -2496,7 +2504,7 @@
         <v>0.5666</v>
       </c>
       <c r="T18" s="7" t="n">
-        <v>7800</v>
+        <v>9770</v>
       </c>
       <c r="U18" s="7" t="n">
         <v>4.3436</v>
@@ -2589,7 +2597,7 @@
         <v>0.4596</v>
       </c>
       <c r="T19" s="7" t="n">
-        <v>9505</v>
+        <v>11906</v>
       </c>
       <c r="U19" s="7" t="n">
         <v>7.0565</v>
@@ -2779,7 +2787,7 @@
         <v>0.6618000000000001</v>
       </c>
       <c r="T21" s="7" t="n">
-        <v>10674</v>
+        <v>13371</v>
       </c>
       <c r="U21" s="7" t="n">
         <v>5.3087</v>
@@ -3002,7 +3010,7 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>FDR-114</t>
+          <t>FDR-070</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -3163,7 +3171,7 @@
         <v>0.6232</v>
       </c>
       <c r="T25" s="7" t="n">
-        <v>8301</v>
+        <v>10397</v>
       </c>
       <c r="U25" s="7" t="n">
         <v>7.024</v>
@@ -3353,7 +3361,7 @@
         <v>0.4248</v>
       </c>
       <c r="T27" s="7" t="n">
-        <v>9921</v>
+        <v>12427</v>
       </c>
       <c r="U27" s="7" t="n">
         <v>8.0266</v>
@@ -3382,7 +3390,7 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>FDR-114</t>
+          <t>FDR-070</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -3576,7 +3584,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>FDR-114</t>
+          <t>FDR-070</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -3673,7 +3681,7 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>FDR-137</t>
+          <t>FDR-179</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -3683,7 +3691,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
@@ -3697,7 +3705,11 @@
       <c r="F31" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G31" s="7" t="inlineStr"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -3710,7 +3722,7 @@
         <v>92.09999999999999</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L31" s="7" t="n">
         <v>0</v>
@@ -3719,7 +3731,7 @@
         <v>0</v>
       </c>
       <c r="N31" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O31" s="7" t="b">
         <v>0</v>
@@ -3731,13 +3743,13 @@
         <v>0.3539</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S31" s="7" t="n">
         <v>0.4735</v>
       </c>
       <c r="T31" s="7" t="n">
-        <v>9552</v>
+        <v>0</v>
       </c>
       <c r="U31" s="7" t="n">
         <v>7.0908</v>
@@ -3863,7 +3875,7 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>FDR-114</t>
+          <t>FDR-070</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -4024,7 +4036,7 @@
         <v>0.3906</v>
       </c>
       <c r="T34" s="7" t="n">
-        <v>11337</v>
+        <v>14201</v>
       </c>
       <c r="U34" s="7" t="n">
         <v>5.8913</v>
@@ -4150,7 +4162,7 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>FDR-008</t>
+          <t>FDR-006</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -4160,7 +4172,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D36" s="7" t="n">
@@ -4174,7 +4186,11 @@
       <c r="F36" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G36" s="7" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -4187,7 +4203,7 @@
         <v>115.3</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L36" s="7" t="n">
         <v>0</v>
@@ -4196,7 +4212,7 @@
         <v>0</v>
       </c>
       <c r="N36" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O36" s="7" t="b">
         <v>0</v>
@@ -4208,13 +4224,13 @@
         <v>0.1392</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S36" s="7" t="n">
         <v>0.3906</v>
       </c>
       <c r="T36" s="7" t="n">
-        <v>11337</v>
+        <v>0</v>
       </c>
       <c r="U36" s="7" t="n">
         <v>5.8913</v>
@@ -4404,7 +4420,7 @@
         <v>0.6744</v>
       </c>
       <c r="T38" s="7" t="n">
-        <v>11785</v>
+        <v>14762</v>
       </c>
       <c r="U38" s="7" t="n">
         <v>5.0155</v>
@@ -4497,7 +4513,7 @@
         <v>1</v>
       </c>
       <c r="T39" s="7" t="n">
-        <v>51299</v>
+        <v>64259</v>
       </c>
       <c r="U39" s="7" t="n">
         <v>1.1425</v>
@@ -4590,7 +4606,7 @@
         <v>0.8004</v>
       </c>
       <c r="T40" s="7" t="n">
-        <v>14266</v>
+        <v>17870</v>
       </c>
       <c r="U40" s="7" t="n">
         <v>4.5541</v>
@@ -4780,7 +4796,7 @@
         <v>0.5669999999999999</v>
       </c>
       <c r="T42" s="7" t="n">
-        <v>10064</v>
+        <v>12606</v>
       </c>
       <c r="U42" s="7" t="n">
         <v>6.2014</v>
@@ -4970,7 +4986,7 @@
         <v>0.4452</v>
       </c>
       <c r="T44" s="7" t="n">
-        <v>9214</v>
+        <v>11541</v>
       </c>
       <c r="U44" s="7" t="n">
         <v>3.8304</v>
@@ -5160,7 +5176,7 @@
         <v>0.424</v>
       </c>
       <c r="T46" s="7" t="n">
-        <v>11015</v>
+        <v>13798</v>
       </c>
       <c r="U46" s="7" t="n">
         <v>7.3596</v>
@@ -5447,7 +5463,7 @@
         <v>0.6186</v>
       </c>
       <c r="T49" s="7" t="n">
-        <v>7591</v>
+        <v>9509</v>
       </c>
       <c r="U49" s="7" t="n">
         <v>4.6584</v>
@@ -5767,7 +5783,7 @@
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>FDR-346</t>
+          <t>FDR-345</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -5777,7 +5793,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
@@ -5791,7 +5807,11 @@
       <c r="F53" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G53" s="7" t="inlineStr"/>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
           <t>HP</t>
@@ -5804,13 +5824,13 @@
         <v>12.6</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M53" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N53" s="7" t="n">
         <v>0</v>
@@ -5825,13 +5845,13 @@
         <v>1</v>
       </c>
       <c r="R53" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S53" s="7" t="n">
         <v>1</v>
       </c>
       <c r="T53" s="7" t="n">
-        <v>51299</v>
+        <v>0</v>
       </c>
       <c r="U53" s="7" t="n">
         <v>1.1425</v>
@@ -5924,7 +5944,7 @@
         <v>0.5866</v>
       </c>
       <c r="T54" s="7" t="n">
-        <v>8298</v>
+        <v>10394</v>
       </c>
       <c r="U54" s="7" t="n">
         <v>7.0213</v>
@@ -5953,7 +5973,7 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>FDR-346</t>
+          <t>FDR-345</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -6050,7 +6070,7 @@
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>FDR-346</t>
+          <t>FDR-345</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -6147,7 +6167,7 @@
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>FDR-346</t>
+          <t>FDR-345</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -6308,7 +6328,7 @@
         <v>0.5318000000000001</v>
       </c>
       <c r="T58" s="7" t="n">
-        <v>10506</v>
+        <v>13160</v>
       </c>
       <c r="U58" s="7" t="n">
         <v>6.057</v>
@@ -7177,7 +7197,7 @@
         <v>0.4824</v>
       </c>
       <c r="T67" s="7" t="n">
-        <v>10754</v>
+        <v>13471</v>
       </c>
       <c r="U67" s="7" t="n">
         <v>6.1465</v>
@@ -7206,7 +7226,7 @@
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>FDR-131</t>
+          <t>FDR-125</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -7216,7 +7236,7 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D68" s="7" t="n">
@@ -7230,7 +7250,11 @@
       <c r="F68" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G68" s="7" t="inlineStr"/>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -7243,7 +7267,7 @@
         <v>101.2</v>
       </c>
       <c r="K68" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L68" s="7" t="n">
         <v>0</v>
@@ -7252,7 +7276,7 @@
         <v>0</v>
       </c>
       <c r="N68" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O68" s="7" t="b">
         <v>0</v>
@@ -7264,13 +7288,13 @@
         <v>0.2771</v>
       </c>
       <c r="R68" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S68" s="7" t="n">
         <v>0.5318000000000001</v>
       </c>
       <c r="T68" s="7" t="n">
-        <v>10506</v>
+        <v>0</v>
       </c>
       <c r="U68" s="7" t="n">
         <v>6.057</v>
@@ -7460,7 +7484,7 @@
         <v>0.2222</v>
       </c>
       <c r="T70" s="7" t="n">
-        <v>10801</v>
+        <v>13529</v>
       </c>
       <c r="U70" s="7" t="n">
         <v>5.2923</v>
@@ -7553,7 +7577,7 @@
         <v>0.6173999999999999</v>
       </c>
       <c r="T71" s="7" t="n">
-        <v>8116</v>
+        <v>10167</v>
       </c>
       <c r="U71" s="7" t="n">
         <v>6.5076</v>
@@ -7582,7 +7606,7 @@
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>FDR-194</t>
+          <t>FDR-193</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -7592,7 +7616,7 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D72" s="7" t="n">
@@ -7606,7 +7630,11 @@
       <c r="F72" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G72" s="7" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
           <t>HP</t>
@@ -7619,13 +7647,13 @@
         <v>106.2</v>
       </c>
       <c r="K72" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L72" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M72" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N72" s="7" t="n">
         <v>0</v>
@@ -7640,13 +7668,13 @@
         <v>0.4253</v>
       </c>
       <c r="R72" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S72" s="7" t="n">
         <v>0.6173999999999999</v>
       </c>
       <c r="T72" s="7" t="n">
-        <v>8116</v>
+        <v>0</v>
       </c>
       <c r="U72" s="7" t="n">
         <v>6.5076</v>
@@ -7933,7 +7961,7 @@
         <v>0.2762</v>
       </c>
       <c r="T75" s="7" t="n">
-        <v>13603</v>
+        <v>17040</v>
       </c>
       <c r="U75" s="7" t="n">
         <v>5.5881</v>
@@ -8166,7 +8194,7 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>UPGRADED_TO_TRUNK</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D78" s="7" t="n">
@@ -8180,32 +8208,36 @@
       <c r="F78" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G78" s="7" t="inlineStr"/>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="I78" s="7" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>87.2</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M78" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="O78" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P78" s="7" t="n">
         <v>0.4598</v>
@@ -8220,7 +8252,7 @@
         <v>0.2762</v>
       </c>
       <c r="T78" s="7" t="n">
-        <v>13603</v>
+        <v>0</v>
       </c>
       <c r="U78" s="7" t="n">
         <v>5.5881</v>
@@ -8259,7 +8291,7 @@
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>UPGRADED_TO_TRUNK</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D79" s="7" t="n">
@@ -8273,32 +8305,36 @@
       <c r="F79" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G79" s="7" t="inlineStr"/>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="I79" s="7" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>87.2</v>
       </c>
       <c r="K79" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L79" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M79" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N79" s="7" t="n">
         <v>0</v>
       </c>
       <c r="O79" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P79" s="7" t="n">
         <v>0.4598</v>
@@ -8313,7 +8349,7 @@
         <v>0.2762</v>
       </c>
       <c r="T79" s="7" t="n">
-        <v>13603</v>
+        <v>0</v>
       </c>
       <c r="U79" s="7" t="n">
         <v>5.5881</v>
@@ -8449,7 +8485,7 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>UPGRADED_TO_TRUNK</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D81" s="7" t="n">
@@ -8463,32 +8499,36 @@
       <c r="F81" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G81" s="7" t="inlineStr"/>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="I81" s="7" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>101.8</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L81" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M81" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N81" s="7" t="n">
         <v>0</v>
       </c>
       <c r="O81" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P81" s="7" t="n">
         <v>0.5874</v>
@@ -8503,7 +8543,7 @@
         <v>0.4374</v>
       </c>
       <c r="T81" s="7" t="n">
-        <v>9978</v>
+        <v>0</v>
       </c>
       <c r="U81" s="7" t="n">
         <v>5.1108</v>
@@ -8542,7 +8582,7 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>UPGRADED_TO_TRUNK</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D82" s="7" t="n">
@@ -8556,32 +8596,36 @@
       <c r="F82" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G82" s="7" t="inlineStr"/>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="I82" s="7" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>101.8</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M82" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="O82" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P82" s="7" t="n">
         <v>0.5874</v>
@@ -8596,7 +8640,7 @@
         <v>0.4374</v>
       </c>
       <c r="T82" s="7" t="n">
-        <v>9978</v>
+        <v>0</v>
       </c>
       <c r="U82" s="7" t="n">
         <v>5.1108</v>
@@ -8635,7 +8679,7 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>UPGRADED_TO_TRUNK</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D83" s="7" t="n">
@@ -8649,32 +8693,36 @@
       <c r="F83" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G83" s="7" t="inlineStr"/>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="I83" s="7" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="J83" s="7" t="n">
         <v>101.8</v>
       </c>
       <c r="K83" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L83" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M83" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N83" s="7" t="n">
         <v>0</v>
       </c>
       <c r="O83" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P83" s="7" t="n">
         <v>0.5874</v>
@@ -8689,7 +8737,7 @@
         <v>0.4374</v>
       </c>
       <c r="T83" s="7" t="n">
-        <v>9978</v>
+        <v>0</v>
       </c>
       <c r="U83" s="7" t="n">
         <v>5.1108</v>
@@ -9009,7 +9057,7 @@
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -9019,7 +9067,7 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D87" s="7" t="n">
@@ -9033,7 +9081,11 @@
       <c r="F87" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G87" s="7" t="inlineStr"/>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H87" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -9046,13 +9098,13 @@
         <v>106.5</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L87" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M87" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N87" s="7" t="n">
         <v>0</v>
@@ -9067,13 +9119,13 @@
         <v>0.274</v>
       </c>
       <c r="R87" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S87" s="7" t="n">
         <v>0.4248</v>
       </c>
       <c r="T87" s="7" t="n">
-        <v>9921</v>
+        <v>0</v>
       </c>
       <c r="U87" s="7" t="n">
         <v>8.0266</v>
@@ -9490,7 +9542,7 @@
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -9684,7 +9736,7 @@
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -9694,7 +9746,7 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D94" s="7" t="n">
@@ -9708,10 +9760,14 @@
       <c r="F94" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G94" s="7" t="inlineStr"/>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H94" s="7" t="inlineStr">
         <is>
-          <t>LP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="I94" s="7" t="n">
@@ -9721,13 +9777,13 @@
         <v>89.90000000000001</v>
       </c>
       <c r="K94" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L94" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M94" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N94" s="7" t="n">
         <v>0</v>
@@ -9742,13 +9798,13 @@
         <v>0.0929</v>
       </c>
       <c r="R94" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S94" s="7" t="n">
         <v>0.2841</v>
       </c>
       <c r="T94" s="7" t="n">
-        <v>14362</v>
+        <v>0</v>
       </c>
       <c r="U94" s="7" t="n">
         <v>5.8992</v>
@@ -10132,7 +10188,7 @@
         <v>0.466</v>
       </c>
       <c r="T98" s="7" t="n">
-        <v>8801</v>
+        <v>11024</v>
       </c>
       <c r="U98" s="7" t="n">
         <v>6.0104</v>
@@ -10258,7 +10314,7 @@
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -10355,7 +10411,7 @@
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -10452,7 +10508,7 @@
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -10807,7 +10863,7 @@
         <v>0.386</v>
       </c>
       <c r="T105" s="7" t="n">
-        <v>7071</v>
+        <v>8857</v>
       </c>
       <c r="U105" s="7" t="n">
         <v>4.7414</v>
@@ -11224,7 +11280,7 @@
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
@@ -11321,7 +11377,7 @@
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
@@ -11515,7 +11571,7 @@
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
@@ -11676,7 +11732,7 @@
         <v>0.3943</v>
       </c>
       <c r="T114" s="7" t="n">
-        <v>6923</v>
+        <v>8671</v>
       </c>
       <c r="U114" s="7" t="n">
         <v>4.643</v>
@@ -11802,7 +11858,7 @@
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -11963,7 +12019,7 @@
         <v>0.549</v>
       </c>
       <c r="T117" s="7" t="n">
-        <v>7720</v>
+        <v>9671</v>
       </c>
       <c r="U117" s="7" t="n">
         <v>6.1122</v>
@@ -11992,7 +12048,7 @@
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>FDR-111</t>
+          <t>FDR-108</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -12002,7 +12058,7 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D118" s="7" t="n">
@@ -12016,7 +12072,11 @@
       <c r="F118" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G118" s="7" t="inlineStr"/>
+      <c r="G118" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H118" s="7" t="inlineStr">
         <is>
           <t>HP</t>
@@ -12029,7 +12089,7 @@
         <v>70.8</v>
       </c>
       <c r="K118" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L118" s="7" t="n">
         <v>0</v>
@@ -12038,7 +12098,7 @@
         <v>0</v>
       </c>
       <c r="N118" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O118" s="7" t="b">
         <v>0</v>
@@ -12050,13 +12110,13 @@
         <v>0.3521</v>
       </c>
       <c r="R118" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S118" s="7" t="n">
         <v>0.6186</v>
       </c>
       <c r="T118" s="7" t="n">
-        <v>7591</v>
+        <v>0</v>
       </c>
       <c r="U118" s="7" t="n">
         <v>4.6584</v>
@@ -12246,7 +12306,7 @@
         <v>0.3846</v>
       </c>
       <c r="T120" s="7" t="n">
-        <v>14811</v>
+        <v>18552</v>
       </c>
       <c r="U120" s="7" t="n">
         <v>5.3506</v>
@@ -13245,7 +13305,7 @@
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
@@ -13342,7 +13402,7 @@
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
@@ -13439,7 +13499,7 @@
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
         <is>
-          <t>FDR-209</t>
+          <t>FDR-205</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
@@ -13449,7 +13509,7 @@
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D133" s="7" t="n">
@@ -13463,7 +13523,11 @@
       <c r="F133" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G133" s="7" t="inlineStr"/>
+      <c r="G133" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -13476,7 +13540,7 @@
         <v>101.1</v>
       </c>
       <c r="K133" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L133" s="7" t="n">
         <v>0</v>
@@ -13485,7 +13549,7 @@
         <v>0</v>
       </c>
       <c r="N133" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O133" s="7" t="b">
         <v>0</v>
@@ -13497,13 +13561,13 @@
         <v>0.302</v>
       </c>
       <c r="R133" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S133" s="7" t="n">
         <v>0.549</v>
       </c>
       <c r="T133" s="7" t="n">
-        <v>7720</v>
+        <v>0</v>
       </c>
       <c r="U133" s="7" t="n">
         <v>6.1122</v>
@@ -13532,7 +13596,7 @@
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
@@ -13823,7 +13887,7 @@
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -14308,7 +14372,7 @@
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
@@ -14566,7 +14630,7 @@
         <v>0.732</v>
       </c>
       <c r="T144" s="7" t="n">
-        <v>10350</v>
+        <v>12964</v>
       </c>
       <c r="U144" s="7" t="n">
         <v>8.016299999999999</v>
@@ -14659,7 +14723,7 @@
         <v>0.3574</v>
       </c>
       <c r="T145" s="7" t="n">
-        <v>9692</v>
+        <v>12141</v>
       </c>
       <c r="U145" s="7" t="n">
         <v>4.7253</v>
@@ -14688,7 +14752,7 @@
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
@@ -14785,7 +14849,7 @@
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
@@ -14882,7 +14946,7 @@
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
         <is>
-          <t>FDR-188</t>
+          <t>FDR-186</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
@@ -14892,7 +14956,7 @@
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D148" s="7" t="n">
@@ -14906,7 +14970,11 @@
       <c r="F148" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G148" s="7" t="inlineStr"/>
+      <c r="G148" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H148" s="7" t="inlineStr">
         <is>
           <t>LP</t>
@@ -14919,13 +14987,13 @@
         <v>78.90000000000001</v>
       </c>
       <c r="K148" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L148" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M148" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N148" s="7" t="n">
         <v>0</v>
@@ -14940,13 +15008,13 @@
         <v>0.1234</v>
       </c>
       <c r="R148" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S148" s="7" t="n">
         <v>0.177</v>
       </c>
       <c r="T148" s="7" t="n">
-        <v>10688</v>
+        <v>0</v>
       </c>
       <c r="U148" s="7" t="n">
         <v>2.0631</v>
@@ -15072,7 +15140,7 @@
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
@@ -15330,7 +15398,7 @@
         <v>0.3803</v>
       </c>
       <c r="T152" s="7" t="n">
-        <v>8375</v>
+        <v>10490</v>
       </c>
       <c r="U152" s="7" t="n">
         <v>5.617</v>
@@ -15423,7 +15491,7 @@
         <v>0.8052</v>
       </c>
       <c r="T153" s="7" t="n">
-        <v>4843</v>
+        <v>6067</v>
       </c>
       <c r="U153" s="7" t="n">
         <v>2.5893</v>
@@ -15452,7 +15520,7 @@
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B154" s="7" t="inlineStr">
@@ -15549,7 +15617,7 @@
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
         <is>
-          <t>FDR-092</t>
+          <t>FDR-090</t>
         </is>
       </c>
       <c r="B155" s="7" t="inlineStr">
@@ -15559,7 +15627,7 @@
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D155" s="7" t="n">
@@ -15573,7 +15641,11 @@
       <c r="F155" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G155" s="7" t="inlineStr"/>
+      <c r="G155" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
           <t>HP</t>
@@ -15586,7 +15658,7 @@
         <v>67.5</v>
       </c>
       <c r="K155" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L155" s="7" t="n">
         <v>0</v>
@@ -15595,7 +15667,7 @@
         <v>0</v>
       </c>
       <c r="N155" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O155" s="7" t="b">
         <v>0</v>
@@ -15607,13 +15679,13 @@
         <v>0.4545</v>
       </c>
       <c r="R155" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S155" s="7" t="n">
         <v>0.7272</v>
       </c>
       <c r="T155" s="7" t="n">
-        <v>7514</v>
+        <v>0</v>
       </c>
       <c r="U155" s="7" t="n">
         <v>5.0024</v>
@@ -15739,7 +15811,7 @@
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
         <is>
-          <t>FDR-153</t>
+          <t>FDR-123</t>
         </is>
       </c>
       <c r="B157" s="7" t="inlineStr">
@@ -15749,7 +15821,7 @@
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D157" s="7" t="n">
@@ -15763,7 +15835,11 @@
       <c r="F157" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G157" s="7" t="inlineStr"/>
+      <c r="G157" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H157" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -15776,7 +15852,7 @@
         <v>66</v>
       </c>
       <c r="K157" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L157" s="7" t="n">
         <v>0</v>
@@ -15785,7 +15861,7 @@
         <v>0</v>
       </c>
       <c r="N157" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O157" s="7" t="b">
         <v>0</v>
@@ -15797,13 +15873,13 @@
         <v>0.2912</v>
       </c>
       <c r="R157" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S157" s="7" t="n">
         <v>0.4662</v>
       </c>
       <c r="T157" s="7" t="n">
-        <v>7057</v>
+        <v>0</v>
       </c>
       <c r="U157" s="7" t="n">
         <v>3.3704</v>
@@ -15896,7 +15972,7 @@
         <v>0.5376</v>
       </c>
       <c r="T158" s="7" t="n">
-        <v>7803</v>
+        <v>9774</v>
       </c>
       <c r="U158" s="7" t="n">
         <v>4.3834</v>
@@ -16022,7 +16098,7 @@
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
         <is>
-          <t>FDR-153</t>
+          <t>FDR-123</t>
         </is>
       </c>
       <c r="B160" s="7" t="inlineStr">
@@ -16119,7 +16195,7 @@
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B161" s="7" t="inlineStr">
@@ -16701,7 +16777,7 @@
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B167" s="7" t="inlineStr">
@@ -17186,7 +17262,7 @@
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
         <is>
-          <t>FDR-014</t>
+          <t>FDR-012</t>
         </is>
       </c>
       <c r="B172" s="7" t="inlineStr">
@@ -17196,7 +17272,7 @@
       </c>
       <c r="C172" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D172" s="7" t="n">
@@ -17210,7 +17286,11 @@
       <c r="F172" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G172" s="7" t="inlineStr"/>
+      <c r="G172" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H172" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -17223,7 +17303,7 @@
         <v>89.7</v>
       </c>
       <c r="K172" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L172" s="7" t="n">
         <v>0</v>
@@ -17232,7 +17312,7 @@
         <v>0</v>
       </c>
       <c r="N172" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O172" s="7" t="b">
         <v>0</v>
@@ -17244,13 +17324,13 @@
         <v>0.1523</v>
       </c>
       <c r="R172" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S172" s="7" t="n">
         <v>0.3574</v>
       </c>
       <c r="T172" s="7" t="n">
-        <v>9692</v>
+        <v>0</v>
       </c>
       <c r="U172" s="7" t="n">
         <v>4.7253</v>
@@ -17440,7 +17520,7 @@
         <v>0.4856</v>
       </c>
       <c r="T174" s="7" t="n">
-        <v>5014</v>
+        <v>6281</v>
       </c>
       <c r="U174" s="7" t="n">
         <v>3.6226</v>
@@ -17727,7 +17807,7 @@
         <v>0.6697</v>
       </c>
       <c r="T177" s="7" t="n">
-        <v>7517</v>
+        <v>9416</v>
       </c>
       <c r="U177" s="7" t="n">
         <v>5.6356</v>
@@ -17756,7 +17836,7 @@
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
         <is>
-          <t>FDR-153</t>
+          <t>FDR-123</t>
         </is>
       </c>
       <c r="B178" s="7" t="inlineStr">
@@ -17950,7 +18030,7 @@
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
         <is>
-          <t>FDR-014</t>
+          <t>FDR-012</t>
         </is>
       </c>
       <c r="B180" s="7" t="inlineStr">
@@ -18208,7 +18288,7 @@
         <v>0.7685999999999999</v>
       </c>
       <c r="T182" s="7" t="n">
-        <v>9775</v>
+        <v>12244</v>
       </c>
       <c r="U182" s="7" t="n">
         <v>5.6844</v>
@@ -18495,7 +18575,7 @@
         <v>0.3795</v>
       </c>
       <c r="T185" s="7" t="n">
-        <v>9277</v>
+        <v>11620</v>
       </c>
       <c r="U185" s="7" t="n">
         <v>6.9564</v>
@@ -18621,7 +18701,7 @@
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B187" s="7" t="inlineStr">
@@ -19170,7 +19250,7 @@
         <v>0.132</v>
       </c>
       <c r="T192" s="7" t="n">
-        <v>6557</v>
+        <v>8213</v>
       </c>
       <c r="U192" s="7" t="n">
         <v>4.3482</v>
@@ -19199,7 +19279,7 @@
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B193" s="7" t="inlineStr">
@@ -19393,7 +19473,7 @@
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B195" s="7" t="inlineStr">
@@ -19845,7 +19925,7 @@
         <v>0.4179</v>
       </c>
       <c r="T199" s="7" t="n">
-        <v>11026</v>
+        <v>13812</v>
       </c>
       <c r="U199" s="7" t="n">
         <v>8.921900000000001</v>
@@ -20423,7 +20503,7 @@
         <v>0.6244</v>
       </c>
       <c r="T205" s="7" t="n">
-        <v>9645</v>
+        <v>12082</v>
       </c>
       <c r="U205" s="7" t="n">
         <v>7.2316</v>
@@ -20549,7 +20629,7 @@
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B207" s="7" t="inlineStr">
@@ -20646,7 +20726,7 @@
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B208" s="7" t="inlineStr">
@@ -20840,7 +20920,7 @@
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
         <is>
-          <t>FDR-092</t>
+          <t>FDR-090</t>
         </is>
       </c>
       <c r="B210" s="7" t="inlineStr">
@@ -20937,7 +21017,7 @@
     <row r="211">
       <c r="A211" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B211" s="7" t="inlineStr">
@@ -21131,7 +21211,7 @@
     <row r="213">
       <c r="A213" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B213" s="7" t="inlineStr">
@@ -21422,7 +21502,7 @@
     <row r="216">
       <c r="A216" s="7" t="inlineStr">
         <is>
-          <t>FDR-153</t>
+          <t>FDR-123</t>
         </is>
       </c>
       <c r="B216" s="7" t="inlineStr">
@@ -21713,7 +21793,7 @@
     <row r="219">
       <c r="A219" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B219" s="7" t="inlineStr">
@@ -21810,7 +21890,7 @@
     <row r="220">
       <c r="A220" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B220" s="7" t="inlineStr">
@@ -22004,7 +22084,7 @@
     <row r="222">
       <c r="A222" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B222" s="7" t="inlineStr">
@@ -22295,7 +22375,7 @@
     <row r="225">
       <c r="A225" s="7" t="inlineStr">
         <is>
-          <t>FDR-037</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B225" s="7" t="inlineStr">
@@ -22305,7 +22385,7 @@
       </c>
       <c r="C225" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D225" s="7" t="n">
@@ -22319,10 +22399,14 @@
       <c r="F225" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G225" s="7" t="inlineStr"/>
+      <c r="G225" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H225" s="7" t="inlineStr">
         <is>
-          <t>LP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="I225" s="7" t="n">
@@ -22332,7 +22416,7 @@
         <v>87.2</v>
       </c>
       <c r="K225" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L225" s="7" t="n">
         <v>0</v>
@@ -22341,7 +22425,7 @@
         <v>0</v>
       </c>
       <c r="N225" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O225" s="7" t="b">
         <v>0</v>
@@ -22353,13 +22437,13 @@
         <v>0.0926</v>
       </c>
       <c r="R225" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S225" s="7" t="n">
         <v>0.2762</v>
       </c>
       <c r="T225" s="7" t="n">
-        <v>13603</v>
+        <v>0</v>
       </c>
       <c r="U225" s="7" t="n">
         <v>5.5881</v>
@@ -22679,7 +22763,7 @@
     <row r="229">
       <c r="A229" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B229" s="7" t="inlineStr">
@@ -22937,7 +23021,7 @@
         <v>0.6919999999999999</v>
       </c>
       <c r="T231" s="7" t="n">
-        <v>9555</v>
+        <v>11968</v>
       </c>
       <c r="U231" s="7" t="n">
         <v>7.1645</v>
@@ -22966,7 +23050,7 @@
     <row r="232">
       <c r="A232" s="7" t="inlineStr">
         <is>
-          <t>FDR-037</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B232" s="7" t="inlineStr">
@@ -23160,7 +23244,7 @@
     <row r="234">
       <c r="A234" s="7" t="inlineStr">
         <is>
-          <t>FDR-098</t>
+          <t>FDR-096</t>
         </is>
       </c>
       <c r="B234" s="7" t="inlineStr">
@@ -23170,7 +23254,7 @@
       </c>
       <c r="C234" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D234" s="7" t="n">
@@ -23184,7 +23268,11 @@
       <c r="F234" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G234" s="7" t="inlineStr"/>
+      <c r="G234" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H234" s="7" t="inlineStr">
         <is>
           <t>HP</t>
@@ -23197,13 +23285,13 @@
         <v>111.7</v>
       </c>
       <c r="K234" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L234" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M234" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N234" s="7" t="n">
         <v>0</v>
@@ -23218,13 +23306,13 @@
         <v>0.5286</v>
       </c>
       <c r="R234" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S234" s="7" t="n">
         <v>0.6919999999999999</v>
       </c>
       <c r="T234" s="7" t="n">
-        <v>9555</v>
+        <v>0</v>
       </c>
       <c r="U234" s="7" t="n">
         <v>7.1645</v>
@@ -23253,7 +23341,7 @@
     <row r="235">
       <c r="A235" s="7" t="inlineStr">
         <is>
-          <t>FDR-021</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B235" s="7" t="inlineStr">
@@ -23350,7 +23438,7 @@
     <row r="236">
       <c r="A236" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B236" s="7" t="inlineStr">
@@ -23447,7 +23535,7 @@
     <row r="237">
       <c r="A237" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B237" s="7" t="inlineStr">
@@ -23641,7 +23729,7 @@
     <row r="239">
       <c r="A239" s="7" t="inlineStr">
         <is>
-          <t>FDR-251</t>
+          <t>FDR-250</t>
         </is>
       </c>
       <c r="B239" s="7" t="inlineStr">
@@ -23651,7 +23739,7 @@
       </c>
       <c r="C239" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D239" s="7" t="n">
@@ -23665,7 +23753,11 @@
       <c r="F239" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G239" s="7" t="inlineStr"/>
+      <c r="G239" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H239" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -23678,7 +23770,7 @@
         <v>119.1</v>
       </c>
       <c r="K239" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L239" s="7" t="n">
         <v>0</v>
@@ -23687,7 +23779,7 @@
         <v>0</v>
       </c>
       <c r="N239" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O239" s="7" t="b">
         <v>0</v>
@@ -23699,13 +23791,13 @@
         <v>0.2644</v>
       </c>
       <c r="R239" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S239" s="7" t="n">
         <v>0.4179</v>
       </c>
       <c r="T239" s="7" t="n">
-        <v>11026</v>
+        <v>0</v>
       </c>
       <c r="U239" s="7" t="n">
         <v>8.921900000000001</v>
@@ -24025,7 +24117,7 @@
     <row r="243">
       <c r="A243" s="7" t="inlineStr">
         <is>
-          <t>FDR-037</t>
+          <t>SSCL-04</t>
         </is>
       </c>
       <c r="B243" s="7" t="inlineStr">
@@ -24413,7 +24505,7 @@
     <row r="247">
       <c r="A247" s="7" t="inlineStr">
         <is>
-          <t>FDR-105</t>
+          <t>FDR-104</t>
         </is>
       </c>
       <c r="B247" s="7" t="inlineStr">
@@ -24423,7 +24515,7 @@
       </c>
       <c r="C247" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D247" s="7" t="n">
@@ -24437,7 +24529,11 @@
       <c r="F247" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G247" s="7" t="inlineStr"/>
+      <c r="G247" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H247" s="7" t="inlineStr">
         <is>
           <t>HP</t>
@@ -24450,7 +24546,7 @@
         <v>73.40000000000001</v>
       </c>
       <c r="K247" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L247" s="7" t="n">
         <v>0</v>
@@ -24459,7 +24555,7 @@
         <v>0</v>
       </c>
       <c r="N247" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O247" s="7" t="b">
         <v>0</v>
@@ -24471,13 +24567,13 @@
         <v>0.332</v>
       </c>
       <c r="R247" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S247" s="7" t="n">
         <v>0.6618000000000001</v>
       </c>
       <c r="T247" s="7" t="n">
-        <v>10674</v>
+        <v>0</v>
       </c>
       <c r="U247" s="7" t="n">
         <v>5.3087</v>
@@ -25670,7 +25766,7 @@
     <row r="260">
       <c r="A260" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B260" s="7" t="inlineStr">
@@ -25961,7 +26057,7 @@
     <row r="263">
       <c r="A263" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B263" s="7" t="inlineStr">
@@ -26349,7 +26445,7 @@
     <row r="267">
       <c r="A267" s="7" t="inlineStr">
         <is>
-          <t>FDR-275</t>
+          <t>FDR-260</t>
         </is>
       </c>
       <c r="B267" s="7" t="inlineStr">
@@ -26359,7 +26455,7 @@
       </c>
       <c r="C267" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D267" s="7" t="n">
@@ -26373,7 +26469,11 @@
       <c r="F267" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G267" s="7" t="inlineStr"/>
+      <c r="G267" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H267" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -26386,7 +26486,7 @@
         <v>79.3</v>
       </c>
       <c r="K267" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L267" s="7" t="n">
         <v>0</v>
@@ -26395,7 +26495,7 @@
         <v>0</v>
       </c>
       <c r="N267" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O267" s="7" t="b">
         <v>0</v>
@@ -26407,13 +26507,13 @@
         <v>0.2311</v>
       </c>
       <c r="R267" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S267" s="7" t="n">
         <v>0.3803</v>
       </c>
       <c r="T267" s="7" t="n">
-        <v>8375</v>
+        <v>0</v>
       </c>
       <c r="U267" s="7" t="n">
         <v>5.617</v>
@@ -27185,7 +27285,7 @@
         <v>0.2764</v>
       </c>
       <c r="T275" s="7" t="n">
-        <v>5927</v>
+        <v>7424</v>
       </c>
       <c r="U275" s="7" t="n">
         <v>4.312</v>
@@ -28572,7 +28672,7 @@
     <row r="290">
       <c r="A290" s="7" t="inlineStr">
         <is>
-          <t>FDR-298</t>
+          <t>FDR-300</t>
         </is>
       </c>
       <c r="B290" s="7" t="inlineStr">
@@ -28582,7 +28682,7 @@
       </c>
       <c r="C290" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D290" s="7" t="n">
@@ -28596,7 +28696,11 @@
       <c r="F290" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G290" s="7" t="inlineStr"/>
+      <c r="G290" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H290" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -28609,7 +28713,7 @@
         <v>100.2</v>
       </c>
       <c r="K290" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L290" s="7" t="n">
         <v>0</v>
@@ -28618,7 +28722,7 @@
         <v>0</v>
       </c>
       <c r="N290" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O290" s="7" t="b">
         <v>0</v>
@@ -28630,13 +28734,13 @@
         <v>0.2227</v>
       </c>
       <c r="R290" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S290" s="7" t="n">
         <v>0.3064</v>
       </c>
       <c r="T290" s="7" t="n">
-        <v>7687</v>
+        <v>0</v>
       </c>
       <c r="U290" s="7" t="n">
         <v>5.7448</v>
@@ -29117,7 +29221,7 @@
         <v>0.5923</v>
       </c>
       <c r="T295" s="7" t="n">
-        <v>8936</v>
+        <v>11193</v>
       </c>
       <c r="U295" s="7" t="n">
         <v>5.0416</v>
@@ -29243,7 +29347,7 @@
     <row r="297">
       <c r="A297" s="7" t="inlineStr">
         <is>
-          <t>FDR-227</t>
+          <t>FDR-225</t>
         </is>
       </c>
       <c r="B297" s="7" t="inlineStr">
@@ -29404,7 +29508,7 @@
         <v>0.6686</v>
       </c>
       <c r="T298" s="7" t="n">
-        <v>11158</v>
+        <v>13977</v>
       </c>
       <c r="U298" s="7" t="n">
         <v>5.8534</v>
@@ -29627,7 +29731,7 @@
     <row r="301">
       <c r="A301" s="7" t="inlineStr">
         <is>
-          <t>FDR-323</t>
+          <t>FDR-320</t>
         </is>
       </c>
       <c r="B301" s="7" t="inlineStr">
@@ -29724,7 +29828,7 @@
     <row r="302">
       <c r="A302" s="7" t="inlineStr">
         <is>
-          <t>FDR-323</t>
+          <t>FDR-320</t>
         </is>
       </c>
       <c r="B302" s="7" t="inlineStr">
@@ -30273,7 +30377,7 @@
         <v>0.7538</v>
       </c>
       <c r="T307" s="7" t="n">
-        <v>6925</v>
+        <v>8675</v>
       </c>
       <c r="U307" s="7" t="n">
         <v>5.1925</v>
@@ -30593,7 +30697,7 @@
     <row r="311">
       <c r="A311" s="7" t="inlineStr">
         <is>
-          <t>FDR-323</t>
+          <t>FDR-320</t>
         </is>
       </c>
       <c r="B311" s="7" t="inlineStr">
@@ -30690,7 +30794,7 @@
     <row r="312">
       <c r="A312" s="7" t="inlineStr">
         <is>
-          <t>FDR-323</t>
+          <t>FDR-320</t>
         </is>
       </c>
       <c r="B312" s="7" t="inlineStr">
@@ -30787,7 +30891,7 @@
     <row r="313">
       <c r="A313" s="7" t="inlineStr">
         <is>
-          <t>FDR-188</t>
+          <t>FDR-186</t>
         </is>
       </c>
       <c r="B313" s="7" t="inlineStr">
@@ -30884,7 +30988,7 @@
     <row r="314">
       <c r="A314" s="7" t="inlineStr">
         <is>
-          <t>FDR-188</t>
+          <t>FDR-186</t>
         </is>
       </c>
       <c r="B314" s="7" t="inlineStr">
@@ -31175,7 +31279,7 @@
     <row r="317">
       <c r="A317" s="7" t="inlineStr">
         <is>
-          <t>FDR-105</t>
+          <t>FDR-104</t>
         </is>
       </c>
       <c r="B317" s="7" t="inlineStr">
@@ -31336,7 +31440,7 @@
         <v>0.412</v>
       </c>
       <c r="T318" s="7" t="n">
-        <v>9313</v>
+        <v>11665</v>
       </c>
       <c r="U318" s="7" t="n">
         <v>7.0982</v>
@@ -31365,7 +31469,7 @@
     <row r="319">
       <c r="A319" s="7" t="inlineStr">
         <is>
-          <t>FDR-134</t>
+          <t>FDR-133</t>
         </is>
       </c>
       <c r="B319" s="7" t="inlineStr">
@@ -31375,7 +31479,7 @@
       </c>
       <c r="C319" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D319" s="7" t="n">
@@ -31389,7 +31493,11 @@
       <c r="F319" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="G319" s="7" t="inlineStr"/>
+      <c r="G319" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H319" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -31402,13 +31510,13 @@
         <v>65</v>
       </c>
       <c r="K319" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L319" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M319" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N319" s="7" t="n">
         <v>0</v>
@@ -31423,13 +31531,13 @@
         <v>0.3458</v>
       </c>
       <c r="R319" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S319" s="7" t="n">
         <v>0.527</v>
       </c>
       <c r="T319" s="7" t="n">
-        <v>5985</v>
+        <v>0</v>
       </c>
       <c r="U319" s="7" t="n">
         <v>3.5833</v>
@@ -31458,7 +31566,7 @@
     <row r="320">
       <c r="A320" s="7" t="inlineStr">
         <is>
-          <t>FDR-134</t>
+          <t>FDR-133</t>
         </is>
       </c>
       <c r="B320" s="7" t="inlineStr">
@@ -32428,7 +32536,7 @@
     <row r="330">
       <c r="A330" s="7" t="inlineStr">
         <is>
-          <t>FDR-219</t>
+          <t>FDR-213</t>
         </is>
       </c>
       <c r="B330" s="7" t="inlineStr">
@@ -32438,7 +32546,7 @@
       </c>
       <c r="C330" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D330" s="7" t="n">
@@ -32452,7 +32560,11 @@
       <c r="F330" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G330" s="7" t="inlineStr"/>
+      <c r="G330" s="7" t="inlineStr">
+        <is>
+          <t>LPV / Tempo</t>
+        </is>
+      </c>
       <c r="H330" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -32465,7 +32577,7 @@
         <v>62.1</v>
       </c>
       <c r="K330" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L330" s="7" t="n">
         <v>0</v>
@@ -32474,7 +32586,7 @@
         <v>0</v>
       </c>
       <c r="N330" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O330" s="7" t="b">
         <v>0</v>
@@ -32486,13 +32598,13 @@
         <v>0.2099</v>
       </c>
       <c r="R330" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S330" s="7" t="n">
         <v>0.4856</v>
       </c>
       <c r="T330" s="7" t="n">
-        <v>5014</v>
+        <v>0</v>
       </c>
       <c r="U330" s="7" t="n">
         <v>3.6226</v>
@@ -32812,7 +32924,7 @@
     <row r="334">
       <c r="A334" s="7" t="inlineStr">
         <is>
-          <t>FDR-114</t>
+          <t>FDR-070</t>
         </is>
       </c>
       <c r="B334" s="7" t="inlineStr">
@@ -32909,7 +33021,7 @@
     <row r="335">
       <c r="A335" s="7" t="inlineStr">
         <is>
-          <t>FDR-114</t>
+          <t>FDR-070</t>
         </is>
       </c>
       <c r="B335" s="7" t="inlineStr">
@@ -33006,7 +33118,7 @@
     <row r="336">
       <c r="A336" s="7" t="inlineStr">
         <is>
-          <t>FDR-211</t>
+          <t>FDR-205</t>
         </is>
       </c>
       <c r="B336" s="7" t="inlineStr">
@@ -33016,7 +33128,7 @@
       </c>
       <c r="C336" s="7" t="inlineStr">
         <is>
-          <t>RETAINED_AS_FEEDER</t>
+          <t>MERGED_INTO_TRUNK</t>
         </is>
       </c>
       <c r="D336" s="7" t="n">
@@ -33030,7 +33142,11 @@
       <c r="F336" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="G336" s="7" t="inlineStr"/>
+      <c r="G336" s="7" t="inlineStr">
+        <is>
+          <t>Private Minibus</t>
+        </is>
+      </c>
       <c r="H336" s="7" t="inlineStr">
         <is>
           <t>MP</t>
@@ -33043,13 +33159,13 @@
         <v>101.1</v>
       </c>
       <c r="K336" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L336" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M336" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N336" s="7" t="n">
         <v>0</v>
@@ -33064,13 +33180,13 @@
         <v>0.302</v>
       </c>
       <c r="R336" s="7" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="S336" s="7" t="n">
         <v>0.549</v>
       </c>
       <c r="T336" s="7" t="n">
-        <v>7720</v>
+        <v>0</v>
       </c>
       <c r="U336" s="7" t="n">
         <v>6.1122</v>
@@ -33163,7 +33279,7 @@
         <v>0.0998</v>
       </c>
       <c r="T337" s="7" t="n">
-        <v>8389</v>
+        <v>10508</v>
       </c>
       <c r="U337" s="7" t="n">
         <v>3.9437</v>
@@ -33256,7 +33372,7 @@
         <v>0.241</v>
       </c>
       <c r="T338" s="7" t="n">
-        <v>18565</v>
+        <v>23255</v>
       </c>
       <c r="U338" s="7" t="n">
         <v>11.5301</v>
@@ -33349,7 +33465,7 @@
         <v>0.153</v>
       </c>
       <c r="T339" s="7" t="n">
-        <v>11981</v>
+        <v>15007</v>
       </c>
       <c r="U339" s="7" t="n">
         <v>7.4408</v>
@@ -33442,7 +33558,7 @@
         <v>0.0683</v>
       </c>
       <c r="T340" s="7" t="n">
-        <v>10660</v>
+        <v>13353</v>
       </c>
       <c r="U340" s="7" t="n">
         <v>5.0117</v>
@@ -33535,7 +33651,7 @@
         <v>0.011</v>
       </c>
       <c r="T341" s="7" t="n">
-        <v>14717</v>
+        <v>18435</v>
       </c>
       <c r="U341" s="7" t="n">
         <v>6.9195</v>
@@ -33628,7 +33744,7 @@
         <v>0.08119999999999999</v>
       </c>
       <c r="T342" s="7" t="n">
-        <v>14761</v>
+        <v>18490</v>
       </c>
       <c r="U342" s="7" t="n">
         <v>9.205</v>
@@ -33915,7 +34031,7 @@
         <v>0.0564</v>
       </c>
       <c r="T345" s="7" t="n">
-        <v>32069</v>
+        <v>40170</v>
       </c>
       <c r="U345" s="7" t="n">
         <v>6.666</v>
@@ -34008,7 +34124,7 @@
         <v>0.1472</v>
       </c>
       <c r="T346" s="7" t="n">
-        <v>16857</v>
+        <v>21115</v>
       </c>
       <c r="U346" s="7" t="n">
         <v>10.4693</v>
@@ -34198,7 +34314,7 @@
         <v>0.1353</v>
       </c>
       <c r="T348" s="7" t="n">
-        <v>20320</v>
+        <v>25453</v>
       </c>
       <c r="U348" s="7" t="n">
         <v>9.301600000000001</v>
@@ -34291,7 +34407,7 @@
         <v>0.0209</v>
       </c>
       <c r="T349" s="7" t="n">
-        <v>14489</v>
+        <v>18149</v>
       </c>
       <c r="U349" s="7" t="n">
         <v>6.8123</v>
@@ -34384,7 +34500,7 @@
         <v>0.0164</v>
       </c>
       <c r="T350" s="7" t="n">
-        <v>13482</v>
+        <v>16888</v>
       </c>
       <c r="U350" s="7" t="n">
         <v>6.3388</v>
@@ -34477,7 +34593,7 @@
         <v>0.2224</v>
       </c>
       <c r="T351" s="7" t="n">
-        <v>15410</v>
+        <v>19303</v>
       </c>
       <c r="U351" s="7" t="n">
         <v>7.0542</v>
@@ -34667,7 +34783,7 @@
         <v>0.1926</v>
       </c>
       <c r="T353" s="7" t="n">
-        <v>9750</v>
+        <v>12213</v>
       </c>
       <c r="U353" s="7" t="n">
         <v>4.5593</v>
@@ -34857,7 +34973,7 @@
         <v>0.6908</v>
       </c>
       <c r="T355" s="7" t="n">
-        <v>9610</v>
+        <v>12037</v>
       </c>
       <c r="U355" s="7" t="n">
         <v>4.3998</v>
@@ -34950,7 +35066,7 @@
         <v>0.598</v>
       </c>
       <c r="T356" s="7" t="n">
-        <v>7299</v>
+        <v>9143</v>
       </c>
       <c r="U356" s="7" t="n">
         <v>4.1003</v>
@@ -35237,7 +35353,7 @@
         <v>0.7554999999999999</v>
       </c>
       <c r="T359" s="7" t="n">
-        <v>7437</v>
+        <v>9316</v>
       </c>
       <c r="U359" s="7" t="n">
         <v>5.411</v>
@@ -35330,7 +35446,7 @@
         <v>0.3425</v>
       </c>
       <c r="T360" s="7" t="n">
-        <v>9029</v>
+        <v>11310</v>
       </c>
       <c r="U360" s="7" t="n">
         <v>4.2225</v>
@@ -35423,7 +35539,7 @@
         <v>0.1884</v>
       </c>
       <c r="T361" s="7" t="n">
-        <v>9535</v>
+        <v>11944</v>
       </c>
       <c r="U361" s="7" t="n">
         <v>5.357</v>
@@ -35613,7 +35729,7 @@
         <v>0.1334</v>
       </c>
       <c r="T363" s="7" t="n">
-        <v>14310</v>
+        <v>17925</v>
       </c>
       <c r="U363" s="7" t="n">
         <v>10.4818</v>
@@ -35706,7 +35822,7 @@
         <v>0.4065</v>
       </c>
       <c r="T364" s="7" t="n">
-        <v>13735</v>
+        <v>17205</v>
       </c>
       <c r="U364" s="7" t="n">
         <v>6.5598</v>
@@ -36381,7 +36497,7 @@
         <v>0.2337</v>
       </c>
       <c r="T371" s="7" t="n">
-        <v>10691</v>
+        <v>13391</v>
       </c>
       <c r="U371" s="7" t="n">
         <v>4.2856</v>
@@ -37153,7 +37269,7 @@
         <v>0.4245</v>
       </c>
       <c r="T379" s="7" t="n">
-        <v>8510</v>
+        <v>10659</v>
       </c>
       <c r="U379" s="7" t="n">
         <v>6.1913</v>
@@ -38313,7 +38429,7 @@
         <v>0.4458</v>
       </c>
       <c r="T391" s="7" t="n">
-        <v>11826</v>
+        <v>14814</v>
       </c>
       <c r="U391" s="7" t="n">
         <v>5.7951</v>
@@ -38406,7 +38522,7 @@
         <v>0.427</v>
       </c>
       <c r="T392" s="7" t="n">
-        <v>16981</v>
+        <v>21270</v>
       </c>
       <c r="U392" s="7" t="n">
         <v>10.2523</v>
@@ -38499,7 +38615,7 @@
         <v>0.2059</v>
       </c>
       <c r="T393" s="7" t="n">
-        <v>8908</v>
+        <v>11159</v>
       </c>
       <c r="U393" s="7" t="n">
         <v>2.0059</v>
@@ -38592,7 +38708,7 @@
         <v>0.5696</v>
       </c>
       <c r="T394" s="7" t="n">
-        <v>8763</v>
+        <v>10976</v>
       </c>
       <c r="U394" s="7" t="n">
         <v>5.9623</v>
@@ -38685,7 +38801,7 @@
         <v>0.131</v>
       </c>
       <c r="T395" s="7" t="n">
-        <v>10545</v>
+        <v>13209</v>
       </c>
       <c r="U395" s="7" t="n">
         <v>2.3745</v>
@@ -38778,7 +38894,7 @@
         <v>0.6685</v>
       </c>
       <c r="T396" s="7" t="n">
-        <v>11098</v>
+        <v>13901</v>
       </c>
       <c r="U396" s="7" t="n">
         <v>5.822</v>
@@ -38871,7 +38987,7 @@
         <v>0.2514</v>
       </c>
       <c r="T397" s="7" t="n">
-        <v>11780</v>
+        <v>14756</v>
       </c>
       <c r="U397" s="7" t="n">
         <v>6.1213</v>
@@ -38964,7 +39080,7 @@
         <v>0.1551</v>
       </c>
       <c r="T398" s="7" t="n">
-        <v>34715</v>
+        <v>43485</v>
       </c>
       <c r="U398" s="7" t="n">
         <v>7.216</v>
@@ -39057,7 +39173,7 @@
         <v>0.0848</v>
       </c>
       <c r="T399" s="7" t="n">
-        <v>12352</v>
+        <v>15472</v>
       </c>
       <c r="U399" s="7" t="n">
         <v>2.7817</v>
@@ -39150,7 +39266,7 @@
         <v>0.5037</v>
       </c>
       <c r="T400" s="7" t="n">
-        <v>9695</v>
+        <v>12144</v>
       </c>
       <c r="U400" s="7" t="n">
         <v>6.8851</v>
@@ -39243,7 +39359,7 @@
         <v>0.2336</v>
       </c>
       <c r="T401" s="7" t="n">
-        <v>12979</v>
+        <v>16258</v>
       </c>
       <c r="U401" s="7" t="n">
         <v>6.7445</v>
@@ -39336,7 +39452,7 @@
         <v>0.9247</v>
       </c>
       <c r="T402" s="7" t="n">
-        <v>4621</v>
+        <v>5788</v>
       </c>
       <c r="U402" s="7" t="n">
         <v>1.0634</v>
@@ -39429,7 +39545,7 @@
         <v>0.6467000000000001</v>
       </c>
       <c r="T403" s="7" t="n">
-        <v>11441</v>
+        <v>14332</v>
       </c>
       <c r="U403" s="7" t="n">
         <v>5.6902</v>
@@ -39522,7 +39638,7 @@
         <v>0.377</v>
       </c>
       <c r="T404" s="7" t="n">
-        <v>16912</v>
+        <v>21184</v>
       </c>
       <c r="U404" s="7" t="n">
         <v>9.164300000000001</v>
@@ -39615,7 +39731,7 @@
         <v>0.273</v>
       </c>
       <c r="T405" s="7" t="n">
-        <v>18749</v>
+        <v>23486</v>
       </c>
       <c r="U405" s="7" t="n">
         <v>7.5619</v>
@@ -39708,7 +39824,7 @@
         <v>0.2234</v>
       </c>
       <c r="T406" s="7" t="n">
-        <v>11606</v>
+        <v>14539</v>
       </c>
       <c r="U406" s="7" t="n">
         <v>7.6963</v>
@@ -39801,7 +39917,7 @@
         <v>0.3254</v>
       </c>
       <c r="T407" s="7" t="n">
-        <v>11411</v>
+        <v>14294</v>
       </c>
       <c r="U407" s="7" t="n">
         <v>4.9129</v>
@@ -39894,7 +40010,7 @@
         <v>0.7244</v>
       </c>
       <c r="T408" s="7" t="n">
-        <v>6213</v>
+        <v>7783</v>
       </c>
       <c r="U408" s="7" t="n">
         <v>2.552</v>
@@ -39987,7 +40103,7 @@
         <v>0.3835</v>
       </c>
       <c r="T409" s="7" t="n">
-        <v>10421</v>
+        <v>13054</v>
       </c>
       <c r="U409" s="7" t="n">
         <v>5.2609</v>
@@ -40080,7 +40196,7 @@
         <v>0.1178</v>
       </c>
       <c r="T410" s="7" t="n">
-        <v>13903</v>
+        <v>17415</v>
       </c>
       <c r="U410" s="7" t="n">
         <v>7.224</v>
@@ -40173,7 +40289,7 @@
         <v>0.0462</v>
       </c>
       <c r="T411" s="7" t="n">
-        <v>16211</v>
+        <v>20306</v>
       </c>
       <c r="U411" s="7" t="n">
         <v>8.4633</v>
@@ -40266,7 +40382,7 @@
         <v>0.3265</v>
       </c>
       <c r="T412" s="7" t="n">
-        <v>20218</v>
+        <v>25325</v>
       </c>
       <c r="U412" s="7" t="n">
         <v>4.4027</v>
@@ -40359,7 +40475,7 @@
         <v>0.2767</v>
       </c>
       <c r="T413" s="7" t="n">
-        <v>13584</v>
+        <v>17016</v>
       </c>
       <c r="U413" s="7" t="n">
         <v>5.849</v>
@@ -40452,7 +40568,7 @@
         <v>0.1632</v>
       </c>
       <c r="T414" s="7" t="n">
-        <v>34599</v>
+        <v>43340</v>
       </c>
       <c r="U414" s="7" t="n">
         <v>6.9352</v>
@@ -40545,7 +40661,7 @@
         <v>0.1397</v>
       </c>
       <c r="T415" s="7" t="n">
-        <v>15226</v>
+        <v>19072</v>
       </c>
       <c r="U415" s="7" t="n">
         <v>7.9121</v>
@@ -40638,7 +40754,7 @@
         <v>0.0876</v>
       </c>
       <c r="T416" s="7" t="n">
-        <v>29539</v>
+        <v>37001</v>
       </c>
       <c r="U416" s="7" t="n">
         <v>6.7975</v>
@@ -40731,7 +40847,7 @@
         <v>0.0336</v>
       </c>
       <c r="T417" s="7" t="n">
-        <v>16354</v>
+        <v>20485</v>
       </c>
       <c r="U417" s="7" t="n">
         <v>7.2435</v>
@@ -40824,7 +40940,7 @@
         <v>0.0344</v>
       </c>
       <c r="T418" s="7" t="n">
-        <v>16062</v>
+        <v>20120</v>
       </c>
       <c r="U418" s="7" t="n">
         <v>7.1149</v>
@@ -40917,7 +41033,7 @@
         <v>0.248</v>
       </c>
       <c r="T419" s="7" t="n">
-        <v>15229</v>
+        <v>19076</v>
       </c>
       <c r="U419" s="7" t="n">
         <v>6.5565</v>
@@ -41010,7 +41126,7 @@
         <v>0.3044</v>
       </c>
       <c r="T420" s="7" t="n">
-        <v>12847</v>
+        <v>16092</v>
       </c>
       <c r="U420" s="7" t="n">
         <v>3.974</v>
@@ -41103,7 +41219,7 @@
         <v>0.0848</v>
       </c>
       <c r="T421" s="7" t="n">
-        <v>12352</v>
+        <v>15472</v>
       </c>
       <c r="U421" s="7" t="n">
         <v>2.7817</v>

</xml_diff>

<commit_message>
kashmir(v3.4.2): Hybrid demand-responsive rural sizing — 924 buses
Sync engine 747fa4e (route-level audit). Rural Regional lifelines are now sized
by demand (35/60/90/120-min, 2-hourly floor) instead of a flat 35-min clock;
Urban/Peri-Urban + SSCL unchanged. Assets regenerated; v3.4.1 workbooks purged.
lib: totalFleet 1144->924 (139/703/82), busesPer1000 0.49->0.40, expansion
91->54; headway-band note + taglines reframed to "city <=35 min; rural lifelines
demand-sized 35-120" (the literal "no route waits >35 min" claim no longer holds
for rural lifelines). Version + download links -> v3.4.2. tsc --noEmit clean.
Plan: 186 active / 924 buses / 30 SSCL / 35.2% coverage of the 6.58M division.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.xlsx
+++ b/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.xlsx
@@ -3797,13 +3797,13 @@
         </is>
       </c>
       <c r="I32" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>136.7</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L32" s="7" t="n">
         <v>0</v>
@@ -3812,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="N32" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O32" s="7" t="b">
         <v>0</v>
@@ -43860,19 +43860,19 @@
         </is>
       </c>
       <c r="I447" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J447" s="7" t="n">
         <v>126.1</v>
       </c>
       <c r="K447" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L447" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M447" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M447" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N447" s="7" t="n">
         <v>0</v>
@@ -43953,19 +43953,19 @@
         </is>
       </c>
       <c r="I448" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J448" s="7" t="n">
         <v>100.8</v>
       </c>
       <c r="K448" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L448" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M448" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N448" s="7" t="n">
         <v>0</v>
@@ -44046,19 +44046,19 @@
         </is>
       </c>
       <c r="I449" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J449" s="7" t="n">
         <v>98.3</v>
       </c>
       <c r="K449" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L449" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M449" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N449" s="7" t="n">
         <v>0</v>
@@ -44139,19 +44139,19 @@
         </is>
       </c>
       <c r="I450" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J450" s="7" t="n">
         <v>132.9</v>
       </c>
       <c r="K450" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L450" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M450" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M450" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N450" s="7" t="n">
         <v>0</v>
@@ -44232,19 +44232,19 @@
         </is>
       </c>
       <c r="I451" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J451" s="7" t="n">
         <v>128.6</v>
       </c>
       <c r="K451" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L451" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M451" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M451" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N451" s="7" t="n">
         <v>0</v>
@@ -44325,19 +44325,19 @@
         </is>
       </c>
       <c r="I452" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J452" s="7" t="n">
         <v>116.8</v>
       </c>
       <c r="K452" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L452" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M452" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N452" s="7" t="n">
         <v>0</v>
@@ -44418,19 +44418,19 @@
         </is>
       </c>
       <c r="I453" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J453" s="7" t="n">
         <v>45.8</v>
       </c>
       <c r="K453" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L453" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M453" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N453" s="7" t="n">
         <v>0</v>
@@ -44511,19 +44511,19 @@
         </is>
       </c>
       <c r="I454" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J454" s="7" t="n">
         <v>319.2</v>
       </c>
       <c r="K454" s="7" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L454" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M454" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="N454" s="7" t="n">
         <v>0</v>
@@ -44701,19 +44701,19 @@
         </is>
       </c>
       <c r="I456" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J456" s="7" t="n">
         <v>76.7</v>
       </c>
       <c r="K456" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L456" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M456" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N456" s="7" t="n">
         <v>0</v>
@@ -44794,19 +44794,19 @@
         </is>
       </c>
       <c r="I457" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J457" s="7" t="n">
         <v>85.40000000000001</v>
       </c>
       <c r="K457" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L457" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M457" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N457" s="7" t="n">
         <v>0</v>
@@ -44887,19 +44887,19 @@
         </is>
       </c>
       <c r="I458" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J458" s="7" t="n">
         <v>113.5</v>
       </c>
       <c r="K458" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L458" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M458" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N458" s="7" t="n">
         <v>0</v>
@@ -44980,19 +44980,19 @@
         </is>
       </c>
       <c r="I459" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J459" s="7" t="n">
         <v>98.59999999999999</v>
       </c>
       <c r="K459" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L459" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M459" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N459" s="7" t="n">
         <v>0</v>
@@ -45073,19 +45073,19 @@
         </is>
       </c>
       <c r="I460" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J460" s="7" t="n">
         <v>84.5</v>
       </c>
       <c r="K460" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L460" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M460" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N460" s="7" t="n">
         <v>0</v>
@@ -45166,19 +45166,19 @@
         </is>
       </c>
       <c r="I461" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J461" s="7" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="K461" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L461" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M461" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N461" s="7" t="n">
         <v>0</v>
@@ -45259,19 +45259,19 @@
         </is>
       </c>
       <c r="I462" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J462" s="7" t="n">
         <v>121.7</v>
       </c>
       <c r="K462" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L462" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M462" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M462" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N462" s="7" t="n">
         <v>0</v>
@@ -45352,19 +45352,19 @@
         </is>
       </c>
       <c r="I463" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J463" s="7" t="n">
         <v>333.5</v>
       </c>
       <c r="K463" s="7" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L463" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M463" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="N463" s="7" t="n">
         <v>0</v>
@@ -45445,19 +45445,19 @@
         </is>
       </c>
       <c r="I464" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J464" s="7" t="n">
         <v>221.3</v>
       </c>
       <c r="K464" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L464" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M464" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N464" s="7" t="n">
         <v>0</v>
@@ -45635,19 +45635,19 @@
         </is>
       </c>
       <c r="I466" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J466" s="7" t="n">
         <v>288.5</v>
       </c>
       <c r="K466" s="7" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="L466" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M466" s="7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N466" s="7" t="n">
         <v>0</v>
@@ -45728,19 +45728,19 @@
         </is>
       </c>
       <c r="I467" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J467" s="7" t="n">
         <v>284.9</v>
       </c>
       <c r="K467" s="7" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="L467" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M467" s="7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N467" s="7" t="n">
         <v>0</v>
@@ -46209,19 +46209,19 @@
         </is>
       </c>
       <c r="I472" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J472" s="7" t="n">
         <v>106.7</v>
       </c>
       <c r="K472" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L472" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M472" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N472" s="7" t="n">
         <v>0</v>
@@ -46302,19 +46302,19 @@
         </is>
       </c>
       <c r="I473" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J473" s="7" t="n">
         <v>91.5</v>
       </c>
       <c r="K473" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L473" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M473" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N473" s="7" t="n">
         <v>0</v>
@@ -46395,19 +46395,19 @@
         </is>
       </c>
       <c r="I474" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J474" s="7" t="n">
         <v>98.90000000000001</v>
       </c>
       <c r="K474" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L474" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M474" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N474" s="7" t="n">
         <v>0</v>
@@ -46488,19 +46488,19 @@
         </is>
       </c>
       <c r="I475" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J475" s="7" t="n">
         <v>85.2</v>
       </c>
       <c r="K475" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L475" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M475" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N475" s="7" t="n">
         <v>0</v>
@@ -46581,19 +46581,19 @@
         </is>
       </c>
       <c r="I476" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J476" s="7" t="n">
         <v>93.7</v>
       </c>
       <c r="K476" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L476" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M476" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N476" s="7" t="n">
         <v>0</v>
@@ -46674,19 +46674,19 @@
         </is>
       </c>
       <c r="I477" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J477" s="7" t="n">
         <v>126.3</v>
       </c>
       <c r="K477" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L477" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M477" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M477" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N477" s="7" t="n">
         <v>0</v>
@@ -46864,19 +46864,19 @@
         </is>
       </c>
       <c r="I479" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J479" s="7" t="n">
         <v>150</v>
       </c>
       <c r="K479" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L479" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M479" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M479" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N479" s="7" t="n">
         <v>0</v>
@@ -47054,19 +47054,19 @@
         </is>
       </c>
       <c r="I481" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J481" s="7" t="n">
         <v>131.9</v>
       </c>
       <c r="K481" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L481" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M481" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M481" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N481" s="7" t="n">
         <v>0</v>
@@ -47147,19 +47147,19 @@
         </is>
       </c>
       <c r="I482" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J482" s="7" t="n">
         <v>118.5</v>
       </c>
       <c r="K482" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L482" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M482" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N482" s="7" t="n">
         <v>0</v>
@@ -47240,19 +47240,19 @@
         </is>
       </c>
       <c r="I483" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J483" s="7" t="n">
         <v>213.1</v>
       </c>
       <c r="K483" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L483" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M483" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N483" s="7" t="n">
         <v>0</v>
@@ -47333,19 +47333,19 @@
         </is>
       </c>
       <c r="I484" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J484" s="7" t="n">
         <v>94.09999999999999</v>
       </c>
       <c r="K484" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L484" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M484" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N484" s="7" t="n">
         <v>0</v>
@@ -47426,19 +47426,19 @@
         </is>
       </c>
       <c r="I485" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J485" s="7" t="n">
         <v>104</v>
       </c>
       <c r="K485" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L485" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M485" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N485" s="7" t="n">
         <v>0</v>
@@ -47519,19 +47519,19 @@
         </is>
       </c>
       <c r="I486" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J486" s="7" t="n">
         <v>264.4</v>
       </c>
       <c r="K486" s="7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L486" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M486" s="7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N486" s="7" t="n">
         <v>0</v>
@@ -47612,19 +47612,19 @@
         </is>
       </c>
       <c r="I487" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J487" s="7" t="n">
         <v>232.9</v>
       </c>
       <c r="K487" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L487" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M487" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N487" s="7" t="n">
         <v>0</v>
@@ -47705,19 +47705,19 @@
         </is>
       </c>
       <c r="I488" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J488" s="7" t="n">
         <v>362.5</v>
       </c>
       <c r="K488" s="7" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="L488" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M488" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="N488" s="7" t="n">
         <v>0</v>
@@ -47895,19 +47895,19 @@
         </is>
       </c>
       <c r="I490" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J490" s="7" t="n">
         <v>175.8</v>
       </c>
       <c r="K490" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L490" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M490" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N490" s="7" t="n">
         <v>0</v>
@@ -48275,19 +48275,19 @@
         </is>
       </c>
       <c r="I494" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J494" s="7" t="n">
         <v>182.3</v>
       </c>
       <c r="K494" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L494" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M494" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N494" s="7" t="n">
         <v>0</v>
@@ -48655,19 +48655,19 @@
         </is>
       </c>
       <c r="I498" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J498" s="7" t="n">
         <v>150.1</v>
       </c>
       <c r="K498" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L498" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M498" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M498" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N498" s="7" t="n">
         <v>0</v>
@@ -48845,19 +48845,19 @@
         </is>
       </c>
       <c r="I500" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J500" s="7" t="n">
         <v>189.4</v>
       </c>
       <c r="K500" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L500" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M500" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N500" s="7" t="n">
         <v>0</v>
@@ -48938,19 +48938,19 @@
         </is>
       </c>
       <c r="I501" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J501" s="7" t="n">
         <v>186</v>
       </c>
       <c r="K501" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L501" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M501" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N501" s="7" t="n">
         <v>0</v>
@@ -49031,19 +49031,19 @@
         </is>
       </c>
       <c r="I502" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J502" s="7" t="n">
         <v>168.9</v>
       </c>
       <c r="K502" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L502" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M502" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M502" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N502" s="7" t="n">
         <v>0</v>
@@ -49504,19 +49504,19 @@
         </is>
       </c>
       <c r="I507" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J507" s="7" t="n">
         <v>169.5</v>
       </c>
       <c r="K507" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L507" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M507" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M507" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N507" s="7" t="n">
         <v>0</v>
@@ -50074,19 +50074,19 @@
         </is>
       </c>
       <c r="I513" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J513" s="7" t="n">
         <v>308.9</v>
       </c>
       <c r="K513" s="7" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="L513" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M513" s="7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N513" s="7" t="n">
         <v>0</v>
@@ -50167,19 +50167,19 @@
         </is>
       </c>
       <c r="I514" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J514" s="7" t="n">
         <v>315.2</v>
       </c>
       <c r="K514" s="7" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L514" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M514" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="N514" s="7" t="n">
         <v>0</v>
@@ -50551,19 +50551,19 @@
         </is>
       </c>
       <c r="I518" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J518" s="7" t="n">
         <v>145.1</v>
       </c>
       <c r="K518" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L518" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M518" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M518" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N518" s="7" t="n">
         <v>0</v>
@@ -50644,19 +50644,19 @@
         </is>
       </c>
       <c r="I519" s="7" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="J519" s="7" t="n">
         <v>173.3</v>
       </c>
       <c r="K519" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L519" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M519" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M519" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N519" s="7" t="n">
         <v>0</v>
@@ -50737,19 +50737,19 @@
         </is>
       </c>
       <c r="I520" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J520" s="7" t="n">
         <v>146.4</v>
       </c>
       <c r="K520" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L520" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M520" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M520" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N520" s="7" t="n">
         <v>0</v>
@@ -50830,19 +50830,19 @@
         </is>
       </c>
       <c r="I521" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J521" s="7" t="n">
         <v>175.6</v>
       </c>
       <c r="K521" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L521" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M521" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N521" s="7" t="n">
         <v>0</v>
@@ -50923,19 +50923,19 @@
         </is>
       </c>
       <c r="I522" s="7" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="J522" s="7" t="n">
         <v>186.4</v>
       </c>
       <c r="K522" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L522" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M522" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N522" s="7" t="n">
         <v>0</v>
@@ -51016,19 +51016,19 @@
         </is>
       </c>
       <c r="I523" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J523" s="7" t="n">
         <v>200.5</v>
       </c>
       <c r="K523" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L523" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M523" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N523" s="7" t="n">
         <v>0</v>
@@ -51206,19 +51206,19 @@
         </is>
       </c>
       <c r="I525" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J525" s="7" t="n">
         <v>181.9</v>
       </c>
       <c r="K525" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L525" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M525" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N525" s="7" t="n">
         <v>0</v>
@@ -51299,19 +51299,19 @@
         </is>
       </c>
       <c r="I526" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J526" s="7" t="n">
         <v>201.1</v>
       </c>
       <c r="K526" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L526" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M526" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N526" s="7" t="n">
         <v>0</v>
@@ -51392,19 +51392,19 @@
         </is>
       </c>
       <c r="I527" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J527" s="7" t="n">
         <v>207.5</v>
       </c>
       <c r="K527" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L527" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M527" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N527" s="7" t="n">
         <v>0</v>
@@ -51485,19 +51485,19 @@
         </is>
       </c>
       <c r="I528" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J528" s="7" t="n">
         <v>194.8</v>
       </c>
       <c r="K528" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L528" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M528" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N528" s="7" t="n">
         <v>0</v>
@@ -52144,19 +52144,19 @@
         </is>
       </c>
       <c r="I535" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J535" s="7" t="n">
         <v>121.9</v>
       </c>
       <c r="K535" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L535" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M535" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M535" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N535" s="7" t="n">
         <v>0</v>
@@ -52237,19 +52237,19 @@
         </is>
       </c>
       <c r="I536" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J536" s="7" t="n">
         <v>151.1</v>
       </c>
       <c r="K536" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L536" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M536" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M536" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N536" s="7" t="n">
         <v>0</v>
@@ -52621,19 +52621,19 @@
         </is>
       </c>
       <c r="I540" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J540" s="7" t="n">
         <v>134.9</v>
       </c>
       <c r="K540" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L540" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M540" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M540" s="7" t="n">
-        <v>3</v>
       </c>
       <c r="N540" s="7" t="n">
         <v>0</v>
@@ -52811,19 +52811,19 @@
         </is>
       </c>
       <c r="I542" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J542" s="7" t="n">
         <v>177.9</v>
       </c>
       <c r="K542" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L542" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M542" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N542" s="7" t="n">
         <v>0</v>
@@ -53870,19 +53870,19 @@
         </is>
       </c>
       <c r="I553" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J553" s="7" t="n">
         <v>168.3</v>
       </c>
       <c r="K553" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L553" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M553" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M553" s="7" t="n">
-        <v>4</v>
       </c>
       <c r="N553" s="7" t="n">
         <v>0</v>
@@ -53963,19 +53963,19 @@
         </is>
       </c>
       <c r="I554" s="7" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="J554" s="7" t="n">
         <v>195.7</v>
       </c>
       <c r="K554" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L554" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M554" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N554" s="7" t="n">
         <v>0</v>
@@ -54343,19 +54343,19 @@
         </is>
       </c>
       <c r="I558" s="7" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="J558" s="7" t="n">
         <v>241.4</v>
       </c>
       <c r="K558" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L558" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M558" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N558" s="7" t="n">
         <v>0</v>
@@ -54436,19 +54436,19 @@
         </is>
       </c>
       <c r="I559" s="7" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="J559" s="7" t="n">
         <v>221.2</v>
       </c>
       <c r="K559" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L559" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M559" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N559" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
kashmir(v3.4.3): rural wait capped at 50 min — 1,044 buses
Sync engine 618c296. Rural Regional lifelines now run 35/40/45/50-min (hard
50-min max wait, was 120) — service quality over fleet minimisation. Assets
regenerated; v3.4.2 workbooks purged. lib: totalFleet 924->1044 (185/776/83),
busesPer1000 0.40->0.45, expansion 54->74; headway-band note + taglines reframed
to "city <=35 min; rural lifelines 35-50 (50-min max)". Version + links -> v3.4.3.
tsc --noEmit clean. Plan: 186 active / 1,044 buses / 30 SSCL / 35.2% coverage.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.xlsx
+++ b/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.xlsx
@@ -3797,13 +3797,13 @@
         </is>
       </c>
       <c r="I32" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>136.7</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L32" s="7" t="n">
         <v>0</v>
@@ -3812,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="N32" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O32" s="7" t="b">
         <v>0</v>
@@ -43860,16 +43860,16 @@
         </is>
       </c>
       <c r="I447" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J447" s="7" t="n">
         <v>126.1</v>
       </c>
       <c r="K447" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L447" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M447" s="7" t="n">
         <v>2</v>
@@ -43953,19 +43953,19 @@
         </is>
       </c>
       <c r="I448" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J448" s="7" t="n">
         <v>100.8</v>
       </c>
       <c r="K448" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L448" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L448" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="M448" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N448" s="7" t="n">
         <v>0</v>
@@ -44046,19 +44046,19 @@
         </is>
       </c>
       <c r="I449" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J449" s="7" t="n">
         <v>98.3</v>
       </c>
       <c r="K449" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L449" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M449" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N449" s="7" t="n">
         <v>0</v>
@@ -44139,16 +44139,16 @@
         </is>
       </c>
       <c r="I450" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J450" s="7" t="n">
         <v>132.9</v>
       </c>
       <c r="K450" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L450" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M450" s="7" t="n">
         <v>2</v>
@@ -44232,16 +44232,16 @@
         </is>
       </c>
       <c r="I451" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J451" s="7" t="n">
         <v>128.6</v>
       </c>
       <c r="K451" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L451" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M451" s="7" t="n">
         <v>2</v>
@@ -44325,19 +44325,19 @@
         </is>
       </c>
       <c r="I452" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J452" s="7" t="n">
         <v>116.8</v>
       </c>
       <c r="K452" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L452" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L452" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="M452" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N452" s="7" t="n">
         <v>0</v>
@@ -44418,7 +44418,7 @@
         </is>
       </c>
       <c r="I453" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J453" s="7" t="n">
         <v>45.8</v>
@@ -44511,19 +44511,19 @@
         </is>
       </c>
       <c r="I454" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J454" s="7" t="n">
         <v>319.2</v>
       </c>
       <c r="K454" s="7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L454" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M454" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N454" s="7" t="n">
         <v>0</v>
@@ -44701,19 +44701,19 @@
         </is>
       </c>
       <c r="I456" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J456" s="7" t="n">
         <v>76.7</v>
       </c>
       <c r="K456" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L456" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M456" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N456" s="7" t="n">
         <v>0</v>
@@ -44794,19 +44794,19 @@
         </is>
       </c>
       <c r="I457" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J457" s="7" t="n">
         <v>85.40000000000001</v>
       </c>
       <c r="K457" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L457" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M457" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N457" s="7" t="n">
         <v>0</v>
@@ -44887,19 +44887,19 @@
         </is>
       </c>
       <c r="I458" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J458" s="7" t="n">
         <v>113.5</v>
       </c>
       <c r="K458" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L458" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L458" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="M458" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N458" s="7" t="n">
         <v>0</v>
@@ -44980,19 +44980,19 @@
         </is>
       </c>
       <c r="I459" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J459" s="7" t="n">
         <v>98.59999999999999</v>
       </c>
       <c r="K459" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L459" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M459" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N459" s="7" t="n">
         <v>0</v>
@@ -45073,19 +45073,19 @@
         </is>
       </c>
       <c r="I460" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J460" s="7" t="n">
         <v>84.5</v>
       </c>
       <c r="K460" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L460" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M460" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N460" s="7" t="n">
         <v>0</v>
@@ -45166,19 +45166,19 @@
         </is>
       </c>
       <c r="I461" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J461" s="7" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="K461" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L461" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M461" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N461" s="7" t="n">
         <v>0</v>
@@ -45259,16 +45259,16 @@
         </is>
       </c>
       <c r="I462" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J462" s="7" t="n">
         <v>121.7</v>
       </c>
       <c r="K462" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L462" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M462" s="7" t="n">
         <v>2</v>
@@ -45352,19 +45352,19 @@
         </is>
       </c>
       <c r="I463" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J463" s="7" t="n">
         <v>333.5</v>
       </c>
       <c r="K463" s="7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L463" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M463" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N463" s="7" t="n">
         <v>0</v>
@@ -45445,19 +45445,19 @@
         </is>
       </c>
       <c r="I464" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J464" s="7" t="n">
         <v>221.3</v>
       </c>
       <c r="K464" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L464" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M464" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N464" s="7" t="n">
         <v>0</v>
@@ -45635,19 +45635,19 @@
         </is>
       </c>
       <c r="I466" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J466" s="7" t="n">
         <v>288.5</v>
       </c>
       <c r="K466" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="L466" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M466" s="7" t="n">
         <v>4</v>
-      </c>
-      <c r="L466" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M466" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N466" s="7" t="n">
         <v>0</v>
@@ -45728,19 +45728,19 @@
         </is>
       </c>
       <c r="I467" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J467" s="7" t="n">
         <v>284.9</v>
       </c>
       <c r="K467" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="L467" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M467" s="7" t="n">
         <v>4</v>
-      </c>
-      <c r="L467" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M467" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N467" s="7" t="n">
         <v>0</v>
@@ -46209,19 +46209,19 @@
         </is>
       </c>
       <c r="I472" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J472" s="7" t="n">
         <v>106.7</v>
       </c>
       <c r="K472" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L472" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L472" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="M472" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N472" s="7" t="n">
         <v>0</v>
@@ -46302,19 +46302,19 @@
         </is>
       </c>
       <c r="I473" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J473" s="7" t="n">
         <v>91.5</v>
       </c>
       <c r="K473" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L473" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M473" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N473" s="7" t="n">
         <v>0</v>
@@ -46395,19 +46395,19 @@
         </is>
       </c>
       <c r="I474" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J474" s="7" t="n">
         <v>98.90000000000001</v>
       </c>
       <c r="K474" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L474" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M474" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N474" s="7" t="n">
         <v>0</v>
@@ -46488,19 +46488,19 @@
         </is>
       </c>
       <c r="I475" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J475" s="7" t="n">
         <v>85.2</v>
       </c>
       <c r="K475" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L475" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M475" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N475" s="7" t="n">
         <v>0</v>
@@ -46581,19 +46581,19 @@
         </is>
       </c>
       <c r="I476" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J476" s="7" t="n">
         <v>93.7</v>
       </c>
       <c r="K476" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L476" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M476" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N476" s="7" t="n">
         <v>0</v>
@@ -46674,16 +46674,16 @@
         </is>
       </c>
       <c r="I477" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J477" s="7" t="n">
         <v>126.3</v>
       </c>
       <c r="K477" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L477" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M477" s="7" t="n">
         <v>2</v>
@@ -46864,16 +46864,16 @@
         </is>
       </c>
       <c r="I479" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J479" s="7" t="n">
         <v>150</v>
       </c>
       <c r="K479" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L479" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M479" s="7" t="n">
         <v>2</v>
@@ -47054,16 +47054,16 @@
         </is>
       </c>
       <c r="I481" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J481" s="7" t="n">
         <v>131.9</v>
       </c>
       <c r="K481" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L481" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M481" s="7" t="n">
         <v>2</v>
@@ -47147,19 +47147,19 @@
         </is>
       </c>
       <c r="I482" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J482" s="7" t="n">
         <v>118.5</v>
       </c>
       <c r="K482" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L482" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L482" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="M482" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N482" s="7" t="n">
         <v>0</v>
@@ -47240,19 +47240,19 @@
         </is>
       </c>
       <c r="I483" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J483" s="7" t="n">
         <v>213.1</v>
       </c>
       <c r="K483" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L483" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M483" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N483" s="7" t="n">
         <v>0</v>
@@ -47333,19 +47333,19 @@
         </is>
       </c>
       <c r="I484" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J484" s="7" t="n">
         <v>94.09999999999999</v>
       </c>
       <c r="K484" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L484" s="7" t="n">
         <v>1</v>
       </c>
       <c r="M484" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N484" s="7" t="n">
         <v>0</v>
@@ -47426,19 +47426,19 @@
         </is>
       </c>
       <c r="I485" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J485" s="7" t="n">
         <v>104</v>
       </c>
       <c r="K485" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L485" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L485" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="M485" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N485" s="7" t="n">
         <v>0</v>
@@ -47519,19 +47519,19 @@
         </is>
       </c>
       <c r="I486" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J486" s="7" t="n">
         <v>264.4</v>
       </c>
       <c r="K486" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="L486" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M486" s="7" t="n">
         <v>4</v>
-      </c>
-      <c r="L486" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M486" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N486" s="7" t="n">
         <v>0</v>
@@ -47612,19 +47612,19 @@
         </is>
       </c>
       <c r="I487" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J487" s="7" t="n">
         <v>232.9</v>
       </c>
       <c r="K487" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L487" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M487" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N487" s="7" t="n">
         <v>0</v>
@@ -47705,19 +47705,19 @@
         </is>
       </c>
       <c r="I488" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J488" s="7" t="n">
         <v>362.5</v>
       </c>
       <c r="K488" s="7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L488" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M488" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N488" s="7" t="n">
         <v>0</v>
@@ -47895,19 +47895,19 @@
         </is>
       </c>
       <c r="I490" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J490" s="7" t="n">
         <v>175.8</v>
       </c>
       <c r="K490" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L490" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M490" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L490" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M490" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N490" s="7" t="n">
         <v>0</v>
@@ -48275,19 +48275,19 @@
         </is>
       </c>
       <c r="I494" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J494" s="7" t="n">
         <v>182.3</v>
       </c>
       <c r="K494" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L494" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M494" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L494" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M494" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N494" s="7" t="n">
         <v>0</v>
@@ -48655,19 +48655,19 @@
         </is>
       </c>
       <c r="I498" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J498" s="7" t="n">
         <v>150.1</v>
       </c>
       <c r="K498" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L498" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M498" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L498" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M498" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N498" s="7" t="n">
         <v>0</v>
@@ -48845,19 +48845,19 @@
         </is>
       </c>
       <c r="I500" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J500" s="7" t="n">
         <v>189.4</v>
       </c>
       <c r="K500" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L500" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M500" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L500" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M500" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N500" s="7" t="n">
         <v>0</v>
@@ -48938,19 +48938,19 @@
         </is>
       </c>
       <c r="I501" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J501" s="7" t="n">
         <v>186</v>
       </c>
       <c r="K501" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L501" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M501" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L501" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M501" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N501" s="7" t="n">
         <v>0</v>
@@ -49031,19 +49031,19 @@
         </is>
       </c>
       <c r="I502" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J502" s="7" t="n">
         <v>168.9</v>
       </c>
       <c r="K502" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L502" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M502" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L502" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M502" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N502" s="7" t="n">
         <v>0</v>
@@ -49504,19 +49504,19 @@
         </is>
       </c>
       <c r="I507" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J507" s="7" t="n">
         <v>169.5</v>
       </c>
       <c r="K507" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L507" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M507" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L507" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M507" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N507" s="7" t="n">
         <v>0</v>
@@ -50074,19 +50074,19 @@
         </is>
       </c>
       <c r="I513" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J513" s="7" t="n">
         <v>308.9</v>
       </c>
       <c r="K513" s="7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L513" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M513" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N513" s="7" t="n">
         <v>0</v>
@@ -50167,19 +50167,19 @@
         </is>
       </c>
       <c r="I514" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J514" s="7" t="n">
         <v>315.2</v>
       </c>
       <c r="K514" s="7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L514" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M514" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N514" s="7" t="n">
         <v>0</v>
@@ -50551,16 +50551,16 @@
         </is>
       </c>
       <c r="I518" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J518" s="7" t="n">
         <v>145.1</v>
       </c>
       <c r="K518" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L518" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M518" s="7" t="n">
         <v>2</v>
@@ -50644,19 +50644,19 @@
         </is>
       </c>
       <c r="I519" s="7" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="J519" s="7" t="n">
         <v>173.3</v>
       </c>
       <c r="K519" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L519" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M519" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L519" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M519" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N519" s="7" t="n">
         <v>0</v>
@@ -50737,16 +50737,16 @@
         </is>
       </c>
       <c r="I520" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J520" s="7" t="n">
         <v>146.4</v>
       </c>
       <c r="K520" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L520" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M520" s="7" t="n">
         <v>2</v>
@@ -50830,19 +50830,19 @@
         </is>
       </c>
       <c r="I521" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J521" s="7" t="n">
         <v>175.6</v>
       </c>
       <c r="K521" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L521" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M521" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L521" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M521" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N521" s="7" t="n">
         <v>0</v>
@@ -50923,19 +50923,19 @@
         </is>
       </c>
       <c r="I522" s="7" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="J522" s="7" t="n">
         <v>186.4</v>
       </c>
       <c r="K522" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L522" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M522" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N522" s="7" t="n">
         <v>0</v>
@@ -51016,19 +51016,19 @@
         </is>
       </c>
       <c r="I523" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J523" s="7" t="n">
         <v>200.5</v>
       </c>
       <c r="K523" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L523" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M523" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N523" s="7" t="n">
         <v>0</v>
@@ -51206,19 +51206,19 @@
         </is>
       </c>
       <c r="I525" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J525" s="7" t="n">
         <v>181.9</v>
       </c>
       <c r="K525" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L525" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M525" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L525" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M525" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N525" s="7" t="n">
         <v>0</v>
@@ -51299,19 +51299,19 @@
         </is>
       </c>
       <c r="I526" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J526" s="7" t="n">
         <v>201.1</v>
       </c>
       <c r="K526" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L526" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M526" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N526" s="7" t="n">
         <v>0</v>
@@ -51392,19 +51392,19 @@
         </is>
       </c>
       <c r="I527" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J527" s="7" t="n">
         <v>207.5</v>
       </c>
       <c r="K527" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L527" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M527" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N527" s="7" t="n">
         <v>0</v>
@@ -51485,19 +51485,19 @@
         </is>
       </c>
       <c r="I528" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J528" s="7" t="n">
         <v>194.8</v>
       </c>
       <c r="K528" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L528" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M528" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L528" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M528" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N528" s="7" t="n">
         <v>0</v>
@@ -52144,16 +52144,16 @@
         </is>
       </c>
       <c r="I535" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J535" s="7" t="n">
         <v>121.9</v>
       </c>
       <c r="K535" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L535" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M535" s="7" t="n">
         <v>2</v>
@@ -52237,19 +52237,19 @@
         </is>
       </c>
       <c r="I536" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J536" s="7" t="n">
         <v>151.1</v>
       </c>
       <c r="K536" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L536" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M536" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L536" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M536" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N536" s="7" t="n">
         <v>0</v>
@@ -52621,16 +52621,16 @@
         </is>
       </c>
       <c r="I540" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J540" s="7" t="n">
         <v>134.9</v>
       </c>
       <c r="K540" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L540" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M540" s="7" t="n">
         <v>2</v>
@@ -52811,19 +52811,19 @@
         </is>
       </c>
       <c r="I542" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J542" s="7" t="n">
         <v>177.9</v>
       </c>
       <c r="K542" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L542" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M542" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L542" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M542" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N542" s="7" t="n">
         <v>0</v>
@@ -53870,19 +53870,19 @@
         </is>
       </c>
       <c r="I553" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J553" s="7" t="n">
         <v>168.3</v>
       </c>
       <c r="K553" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L553" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M553" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L553" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M553" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N553" s="7" t="n">
         <v>0</v>
@@ -53963,19 +53963,19 @@
         </is>
       </c>
       <c r="I554" s="7" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J554" s="7" t="n">
         <v>195.7</v>
       </c>
       <c r="K554" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L554" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M554" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="L554" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M554" s="7" t="n">
-        <v>2</v>
       </c>
       <c r="N554" s="7" t="n">
         <v>0</v>
@@ -54343,7 +54343,7 @@
         </is>
       </c>
       <c r="I558" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J558" s="7" t="n">
         <v>241.4</v>
@@ -54436,19 +54436,19 @@
         </is>
       </c>
       <c r="I559" s="7" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="J559" s="7" t="n">
         <v>221.2</v>
       </c>
       <c r="K559" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L559" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M559" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N559" s="7" t="n">
         <v>0</v>

</xml_diff>